<commit_message>
fix the text alignment
</commit_message>
<xml_diff>
--- a/assets/data/card_database.xlsx
+++ b/assets/data/card_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Documents/develop/source/FlashCard_js/assets/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EEB74D-4F13-C045-A758-B33E04FD858B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F6B16D-A56B-2F4D-B1B1-B931DA133EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17520" yWindow="4400" windowWidth="33300" windowHeight="23100" xr2:uid="{FED5FAB1-E012-AE40-95CA-4818A17FBF71}"/>
+    <workbookView xWindow="8220" yWindow="2680" windowWidth="33300" windowHeight="23100" xr2:uid="{FED5FAB1-E012-AE40-95CA-4818A17FBF71}"/>
   </bookViews>
   <sheets>
     <sheet name="card_database" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7384" uniqueCount="6550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7392" uniqueCount="6550">
   <si>
     <t>Title</t>
   </si>
@@ -25091,7 +25091,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -25273,12 +25273,6 @@
       <sz val="12"/>
       <color rgb="FF333333"/>
       <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color rgb="FF0F1115"/>
-      <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
     <font>
@@ -25629,7 +25623,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -25644,9 +25638,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
@@ -53048,6 +53039,9 @@
       <c r="A873" s="3" t="s">
         <v>6489</v>
       </c>
+      <c r="B873" t="s">
+        <v>5921</v>
+      </c>
       <c r="C873" s="3" t="s">
         <v>6490</v>
       </c>
@@ -53075,6 +53069,9 @@
       <c r="A874" s="3" t="s">
         <v>6496</v>
       </c>
+      <c r="B874" t="s">
+        <v>5921</v>
+      </c>
       <c r="C874" s="3" t="s">
         <v>6503</v>
       </c>
@@ -53101,6 +53098,9 @@
       <c r="A875" s="3" t="s">
         <v>6504</v>
       </c>
+      <c r="B875" t="s">
+        <v>5921</v>
+      </c>
       <c r="C875" s="3" t="s">
         <v>6510</v>
       </c>
@@ -53128,6 +53128,9 @@
       <c r="A876" s="3" t="s">
         <v>6511</v>
       </c>
+      <c r="B876" t="s">
+        <v>5921</v>
+      </c>
       <c r="C876" s="3" t="s">
         <v>6538</v>
       </c>
@@ -53154,6 +53157,9 @@
       <c r="A877" s="3" t="s">
         <v>6512</v>
       </c>
+      <c r="B877" t="s">
+        <v>5921</v>
+      </c>
       <c r="C877" s="3" t="s">
         <v>6539</v>
       </c>
@@ -53180,6 +53186,9 @@
       <c r="A878" s="3" t="s">
         <v>6513</v>
       </c>
+      <c r="B878" t="s">
+        <v>5921</v>
+      </c>
       <c r="C878" s="3" t="s">
         <v>6540</v>
       </c>
@@ -53207,6 +53216,9 @@
       <c r="A879" s="3" t="s">
         <v>6514</v>
       </c>
+      <c r="B879" t="s">
+        <v>5921</v>
+      </c>
       <c r="C879" s="3" t="s">
         <v>6541</v>
       </c>
@@ -53233,6 +53245,9 @@
       <c r="A880" s="3" t="s">
         <v>6543</v>
       </c>
+      <c r="B880" t="s">
+        <v>5921</v>
+      </c>
       <c r="C880" s="3" t="s">
         <v>6544</v>
       </c>
@@ -53248,7 +53263,7 @@
       <c r="H880" s="2" t="s">
         <v>6546</v>
       </c>
-      <c r="I880" s="10" t="s">
+      <c r="I880" s="2" t="s">
         <v>6548</v>
       </c>
       <c r="J880" t="s">

</xml_diff>